<commit_message>
Villa BOQ: add all chapters (excavation, waterproofing, plumbing, electrical, drywall, furniture, flooring)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsSgWbpRzVonxdBKb16Pi8
</commit_message>
<xml_diff>
--- a/villa_ivgi/villa_ivgi_quantities.xlsx
+++ b/villa_ivgi/villa_ivgi_quantities.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>טיח, ריצוף וצבע לפי חדרים</t>
+          <t>טיח וצבע: שטח קירות לפי חדרים</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -1063,12 +1063,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>הגיליונות שבידינו הם של המהנדס, בלי מחיצות פנים</t>
+          <t>בסיס אדריכלי בגיליון החשמל: קירות, פתחים ושמות חדרים</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>נדרשת תוכנית אדריכלית מלאה</t>
+          <t>נדרש היקף חדר × גובה פחות פתחים; הבסיס קיים, החישוב טרם נבנה</t>
         </is>
       </c>
     </row>
@@ -1242,33 +1242,334 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>נקודות חשמל</t>
+          <t>חפירה לראשי כלונסאות וקורות יסוד</t>
         </is>
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>מ"ק</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>kon7-1 + חתכים A5</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>נדרשים מפלסים ומידות ראשי הכלונסאות (OCR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>שטח גג עליון (קו חיצוני של המעקה)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>מ"ר</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>A3 · שכבת WL, שטח סגור 9.4×11.2 מ׳</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>כולל עובי מעקה. לא כולל גגות נמוכים ומרפסות</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>איטום חדרים רטובים ומרפסות</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>מ"ר</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>חדרים רטובים מהבסיס האדריכלי + A7–A8</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>טרם נמדד</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>כלים סניטריים</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
           <t>יח׳</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>דורש השלמה</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>3 גיליונות חשמל (טקסט אמיתי)</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>נדרש תיוג מקרא ↔ סמל</t>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>שכבות A-SNT/SANIT בגיליון החשמל</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>השכבה קיימת, לא נספרה</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>קווי מים וביוב</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>מ׳</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>אין גיליון אינסטלציה בתיק</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>נדרשת תוכנית אינסטלציה</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>נקודות חשמל לפי סוג (שקעים, מפסקים, גופי תאורה)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>יח׳</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>גיליון חשמל קומת קרקע + מקרא כ-30 סמלים</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>הסמלים בנויים מקווים נפרדים וצריך לאחד לפי קרבה ולהתאים למקרא</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>לוחות חשמל וצנרת</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>יח׳/מ׳</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>גיליונות חשמל</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>טרם נמדד</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>גבס ותקרות</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>תקרות גבס ומונמכות</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>מ"ר</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>שטחי חדרים מגיליון החשמל</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>צריך קריאת סימוני התקרה</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ריהוט</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ריהוט קבוע ונגרות פנים</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>יח׳</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>שכבת FURN בגיליון החשמל (כ-1,000 אלמנטים בקומת קרקע)</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>לא נספר, לא כל הריהוט נכלל בכתב</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>שטח רצפה נטו קומת קרקע (חללים סגורים)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>מ"ר</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>גיליון החשמל, בסיס אדריכלי · זיהוי חללים בקנ"מ 1:50</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>אומת: חדרי שינה נמדדו 10.66 ו-10.03 מול 10.65 ו-10.0 בתוכנית. סלון, מטבח ואוכל חלל פתוח אחד</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pricing, partial bills and CSV/print export screen; lighting count
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MsSgWbpRzVonxdBKb16Pi8
</commit_message>
<xml_diff>
--- a/villa_ivgi/villa_ivgi_quantities.xlsx
+++ b/villa_ivgi/villa_ivgi_quantities.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>kon7-1 · ספירת עיגולים בשכבות fl00/fl00d, מאומת למספור 1–27</t>
+          <t>kon7-1 · ספירת עיגולים בשכבות fl00/fl00d, מאומת למספור 1–27 (27 בסה"כ עם ה-Ø60)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -599,53 +599,51 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>סה"כ כלונסאות</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>27</v>
-      </c>
+          <t>אורך כלונסאות כולל</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>יח׳</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>נמדד</t>
+          <t>מ׳</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>סכום שתי השורות</t>
+          <t>טבלת מפלסים בשולי התוכנית (טקסט וקטורי)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>תואם את מספור הכלונסאות בתוכנית</t>
+          <t>דורש OCR של המפלסים</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>אורך כלונסאות כולל</t>
+          <t>בטון ראשי כלונסאות / יסודות</t>
         </is>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>מ׳</t>
+          <t>מ"ק</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -655,12 +653,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>טבלת מפלסים בשולי התוכנית (טקסט וקטורי)</t>
+          <t>kon7-1, kon7-2</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>דורש OCR של המפלסים</t>
+          <t>יש לקרוא מידות וגבהים מהפרטים</t>
         </is>
       </c>
     </row>
@@ -672,13 +670,13 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>בטון ראשי כלונסאות / יסודות</t>
+          <t>ברזל זיון בכלונסאות וביסודות</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>מ"ק</t>
+          <t>ק"ג</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -688,45 +686,47 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>kon7-1, kon7-2</t>
+          <t>kon7-1 ופרטי זיון</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>יש לקרוא מידות וגבהים מהפרטים</t>
+          <t>דורש OCR של טבלאות הזיון</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ברזל זיון בכלונסאות וביסודות</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
+          <t>קירות קומת קרקע, עובי עד 12 ס"מ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>9.1</v>
+      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ק"ג</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>דורש השלמה</t>
+          <t>מ׳</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>kon7-1 ופרטי זיון</t>
+          <t>A1 · שכבת WL, גוף הקיר לפי עובי</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>דורש OCR של טבלאות הזיון</t>
+          <t>מדידה חלקית: גיליון מהנדס עם קירות נושאים בלבד, פתחים מנוכים</t>
         </is>
       </c>
     </row>
@@ -738,11 +738,11 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>קירות קומת קרקע, עובי עד 12 ס"מ</t>
+          <t>קירות קומת קרקע, עובי 12–17 ס"מ</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>9.1</v>
+        <v>16.1</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -756,12 +756,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>A1 · שכבת WL, גוף הקיר לפי עובי</t>
+          <t>A1 · שכבת WL</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>מדידה חלקית: גיליון מהנדס עם קירות נושאים בלבד, פתחים מנוכים</t>
+          <t>כנ"ל</t>
         </is>
       </c>
     </row>
@@ -773,11 +773,11 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>קירות קומת קרקע, עובי 12–17 ס"מ</t>
+          <t>קירות קומת קרקע, עובי 17–23 ס"מ</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>16.1</v>
+        <v>3.6</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -808,11 +808,11 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>קירות קומת קרקע, עובי 17–23 ס"מ</t>
+          <t>קירות קומת קרקע, עובי מעל 23 ס"מ</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.6</v>
+        <v>23.8</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -843,11 +843,11 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>קירות קומת קרקע, עובי מעל 23 ס"מ</t>
+          <t>קירות קומה א׳ (סה"כ בכל העוביים)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>23.8</v>
+        <v>25</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -861,12 +861,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>A1 · שכבת WL</t>
+          <t>A2 · שכבת WL</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>כנ"ל</t>
+          <t>מדידה חלקית</t>
         </is>
       </c>
     </row>
@@ -878,11 +878,11 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>קירות קומה א׳ (סה"כ בכל העוביים)</t>
+          <t>קירות גג / מעקות (עובי מעל 23)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>25</v>
+        <v>44.8</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -896,47 +896,45 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>A2 · שכבת WL</t>
+          <t>A3 · שכבת WL</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>מדידה חלקית</t>
+          <t>יש לאמת מול חתכים</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>קירות גג / מעקות (עובי מעל 23)</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>44.8</v>
-      </c>
+          <t>אלמנטי בטון בקירות קומת קרקע (בהטצ׳)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>מ׳</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>חלקי</t>
+          <t>מ"ר תכנית</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>A3 · שכבת WL</t>
+          <t>A1 · שכבת fl00h</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>יש לאמת מול חתכים</t>
+          <t>זוהו חלקים אך מילוי ההטצ׳ טרם מחושב</t>
         </is>
       </c>
     </row>
@@ -948,13 +946,13 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>אלמנטי בטון בקירות קומת קרקע (בהטצ׳)</t>
+          <t>תקרות ורצפות בטון</t>
         </is>
       </c>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>מ"ר תכנית</t>
+          <t>מ"ר/מ"ק</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -964,12 +962,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>A1 · שכבת fl00h</t>
+          <t>kon7-4…kon7-7</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>זוהו חלקים אך מילוי ההטצ׳ טרם מחושב</t>
+          <t>נדרש מיפוי שכבות בגיליונות התקרה</t>
         </is>
       </c>
     </row>
@@ -981,13 +979,13 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>תקרות ורצפות בטון</t>
+          <t>עמודים</t>
         </is>
       </c>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>מ"ר/מ"ק</t>
+          <t>יח׳/מ"ק</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -997,30 +995,30 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>kon7-4…kon7-7</t>
+          <t>kon7-1…7</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>נדרש מיפוי שכבות בגיליונות התקרה</t>
+          <t>נדרש זיהוי תגיות</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>09–11</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>עמודים</t>
+          <t>טיח וצבע: שטח קירות לפי חדרים</t>
         </is>
       </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>יח׳/מ"ק</t>
+          <t>מ"ר</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1030,30 +1028,30 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>kon7-1…7</t>
+          <t>בסיס אדריכלי בגיליון החשמל: קירות, פתחים ושמות חדרים</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>נדרש זיהוי תגיות</t>
+          <t>נדרש היקף חדר × גובה פחות פתחים; הבסיס קיים, החישוב טרם נבנה</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09–11</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>טיח וצבע: שטח קירות לפי חדרים</t>
+          <t>דלתות וחלונות (פרטים)</t>
         </is>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>מ"ר</t>
+          <t>יח׳</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1063,30 +1061,30 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>בסיס אדריכלי בגיליון החשמל: קירות, פתחים ושמות חדרים</t>
+          <t>A12, A13 · 24 פרטי דלתות</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>נדרש היקף חדר × גובה פחות פתחים; הבסיס קיים, החישוב טרם נבנה</t>
+          <t>יש לספור לפי תגיות</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>דלתות וחלונות (פרטים)</t>
+          <t>איטום גגות ומרפסות</t>
         </is>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>יח׳</t>
+          <t>מ"ר</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1096,98 +1094,98 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>A12, A13 · 24 פרטי דלתות</t>
+          <t>A7, A8 + תוכנית גג</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>יש לספור לפי תגיות</t>
+          <t>נדרש שטח גג</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>איטום גגות ומרפסות</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n"/>
+          <t>פתחים בחזית צפונית (חלונות ודלתות)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>מ"ר</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>דורש השלמה</t>
+          <t>יח׳</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>A7, A8 + תוכנית גג</t>
+          <t>A4 · שכבת hazit 1-0.05, מימדי מסגרות מהחזית 1:50</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>נדרש שטח גג</t>
+          <t>סה"כ 18.1 מ"ר פתח. חזיתות נוספות לא נקראו בשלמות</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>פתחים בחזית צפונית (חלונות ודלתות)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>3</v>
-      </c>
+          <t>גדרות, שער ופיתוח</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>יח׳</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>חלקי</t>
+          <t>מ׳/מ"ר</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>A4 · שכבת hazit 1-0.05, מימדי מסגרות מהחזית 1:50</t>
+          <t>A6 · תוכנית פיתוח וגדרות</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>סה"כ 18.1 מ"ר פתח. חזיתות נוספות לא נקראו בשלמות</t>
+          <t>טרם נמדד</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>גדרות, שער ופיתוח</t>
+          <t>חתכים: גבהי קומות ועובי תקרות</t>
         </is>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>מ׳/מ"ר</t>
+          <t>מ׳</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1197,30 +1195,30 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>A6 · תוכנית פיתוח וגדרות</t>
+          <t>A5 · 3 חתכים 1:50</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>טרם נמדד</t>
+          <t>המפלסים הם טקסט וקטורי, דורש OCR</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>חתכים: גבהי קומות ועובי תקרות</t>
+          <t>חפירה לראשי כלונסאות וקורות יסוד</t>
         </is>
       </c>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>מ׳</t>
+          <t>מ"ק</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1230,45 +1228,47 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>A5 · 3 חתכים 1:50</t>
+          <t>kon7-1 + חתכים A5</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>המפלסים הם טקסט וקטורי, דורש OCR</t>
+          <t>נדרשים מפלסים ומידות ראשי הכלונסאות (OCR)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>חפירה לראשי כלונסאות וקורות יסוד</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n"/>
+          <t>שטח גג עליון (קו חיצוני של המעקה)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>87.2</v>
+      </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>מ"ק</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>דורש השלמה</t>
+          <t>מ"ר</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>kon7-1 + חתכים A5</t>
+          <t>A3 · שכבת WL, שטח סגור 9.4×11.2 מ׳</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>נדרשים מפלסים ומידות ראשי הכלונסאות (OCR)</t>
+          <t>כולל עובי מעקה. לא כולל גגות נמוכים ומרפסות</t>
         </is>
       </c>
     </row>
@@ -1280,48 +1280,46 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>שטח גג עליון (קו חיצוני של המעקה)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>87.2</v>
-      </c>
+          <t>איטום חדרים רטובים ומרפסות</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
           <t>מ"ר</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>חלקי</t>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>דורש השלמה</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>A3 · שכבת WL, שטח סגור 9.4×11.2 מ׳</t>
+          <t>חדרים רטובים מהבסיס האדריכלי + A7–A8</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>כולל עובי מעקה. לא כולל גגות נמוכים ומרפסות</t>
+          <t>טרם נמדד</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>איטום חדרים רטובים ומרפסות</t>
+          <t>כלים סניטריים</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>מ"ר</t>
+          <t>יח׳</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1331,12 +1329,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>חדרים רטובים מהבסיס האדריכלי + A7–A8</t>
+          <t>שכבות A-SNT/SANIT בגיליון החשמל</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>טרם נמדד</t>
+          <t>השכבה קיימת, לא נספרה</t>
         </is>
       </c>
     </row>
@@ -1348,13 +1346,13 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>כלים סניטריים</t>
+          <t>קווי מים וביוב</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>יח׳</t>
+          <t>מ׳</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1364,45 +1362,47 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>שכבות A-SNT/SANIT בגיליון החשמל</t>
+          <t>אין גיליון אינסטלציה בתיק</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>השכבה קיימת, לא נספרה</t>
+          <t>נדרשת תוכנית אינסטלציה</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>קווי מים וביוב</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n"/>
+          <t>גופי תאורה בתקרה (סמל עיגול עם צלב), קומת קרקע</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>מ׳</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>דורש השלמה</t>
+          <t>יח׳</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>חלקי</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>אין גיליון אינסטלציה בתיק</t>
+          <t>גיליון חשמל קומת קרקע · איחוד קווים לסמלים וספירה</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>נדרשת תוכנית אינסטלציה</t>
+          <t>נספרו רק הסמלים שזוהו בביטחון. קומה א׳ וגג טרם נספרו</t>
         </is>
       </c>
     </row>

</xml_diff>